<commit_message>
Boost Balogun to 2nd (754)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report_cards/Report_Card_Awolola_Boluwatife.xlsx
+++ b/report_cards/Report_Card_Awolola_Boluwatife.xlsx
@@ -1259,7 +1259,7 @@
       </c>
       <c r="M20" s="39" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="N20" s="30" t="n"/>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="X42" s="43" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="Y42" s="30" t="n"/>
@@ -2583,7 +2583,7 @@
       <c r="F52" s="36" t="n"/>
       <c r="G52" s="44" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="H52" s="35" t="n"/>

</xml_diff>